<commit_message>
fix: track frontend_php_backup directory to resolve CI 404 test failures
</commit_message>
<xml_diff>
--- a/backend/automated_tests/comprehensive_test_cases.xlsx
+++ b/backend/automated_tests/comprehensive_test_cases.xlsx
@@ -580,7 +580,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-11 16:24:11 | Engine: Selenium + API Hybrid Test Suite</t>
+          <t>Generated: 2026-06-16 13:54:05 | Engine: Selenium + API Hybrid Test Suite</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>Redirected anonymously to Login page. URL: http://localhost/rct-education-web/frontend/auth/login.php</t>
+          <t>Redirected anonymously to Login page. URL: http://localhost/rct-education-web/frontend_php_backup/auth/login.php</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>Access blocked to /frontend/admin/dashboard.php. Page source verified.</t>
+          <t>Access blocked to /frontend_php_backup/admin/dashboard.php. Page source verified.</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Access blocked to /frontend/admin/patient-detail.php?id=57. Page source verified.</t>
+          <t>Access blocked to /frontend_php_backup/admin/patient-detail.php?id=106. Page source verified.</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="F10" s="15" t="inlineStr">
         <is>
-          <t>Access blocked to /frontend/admin/patients.php. Page source verified.</t>
+          <t>Access blocked to /frontend_php_backup/admin/patients.php. Page source verified.</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>Access blocked to /frontend/admin/attendance.php. Page source verified.</t>
+          <t>Access blocked to /frontend_php_backup/admin/attendance.php. Page source verified.</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="F12" s="15" t="inlineStr">
         <is>
-          <t>Access blocked to /frontend/admin/scores.php. Page source verified.</t>
+          <t>Access blocked to /frontend_php_backup/admin/scores.php. Page source verified.</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>Access blocked to /frontend/admin/consent.php. Page source verified.</t>
+          <t>Access blocked to /frontend_php_backup/admin/consent.php. Page source verified.</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="F20" s="15" t="inlineStr">
         <is>
-          <t>Session ID rotated on login. Before: 6iui73qhhuvh0474ok8n89772c, After: u81ikuddegtpvam20uiticjo73</t>
+          <t>Session ID rotated on login. Before: r6tnsb4acp8oifjinb9v3ekma8, After: v3r76o02gjgn5sp3g3ih3jna4c</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="F27" s="11" t="inlineStr">
         <is>
-          <t>Registered successfully and redirected to patient dashboard. URL: http://localhost/rct-education-web/frontend/patient/dashboard.php</t>
+          <t>Registered successfully and redirected to patient dashboard. URL: http://localhost/rct-education-web/frontend_php_backup/patient/dashboard.php</t>
         </is>
       </c>
       <c r="G27" s="12" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>Log in patient succeeded. Redirected to patient dashboard. URL: http://localhost/rct-education-web/frontend/patient/dashboard.php</t>
+          <t>Log in patient succeeded. Redirected to patient dashboard. URL: http://localhost/rct-education-web/frontend_php_backup/patient/dashboard.php</t>
         </is>
       </c>
       <c r="G33" s="12" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>Logged out successfully and redirected to Login page. URL: http://localhost/rct-education-web/frontend/auth/login.php</t>
+          <t>Logged out successfully and redirected to Login page. URL: http://localhost/rct-education-web/frontend_php_backup/auth/login.php</t>
         </is>
       </c>
       <c r="G37" s="12" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="F41" s="11" t="inlineStr">
         <is>
-          <t>Patient logged in with newly updated credentials post-reset. URL: http://localhost/rct-education-web/frontend/patient/dashboard.php</t>
+          <t>Patient logged in with newly updated credentials post-reset. URL: http://localhost/rct-education-web/frontend_php_backup/patient/dashboard.php</t>
         </is>
       </c>
       <c r="G41" s="12" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="F48" s="15" t="inlineStr">
         <is>
-          <t>Consent submitted successfully. Redirected to: http://localhost/rct-education-web/frontend/patient/satisfaction.php</t>
+          <t>Consent submitted successfully. Redirected to: http://localhost/rct-education-web/frontend_php_backup/patient/satisfaction.php</t>
         </is>
       </c>
       <c r="G48" s="12" t="inlineStr">
@@ -2480,7 +2480,7 @@
       </c>
       <c r="F49" s="11" t="inlineStr">
         <is>
-          <t>App satisfaction survey completed. Redirected back to dashboard. URL: http://localhost/rct-education-web/frontend/patient/dashboard.php</t>
+          <t>App satisfaction survey completed. Redirected back to dashboard. URL: http://localhost/rct-education-web/frontend_php_backup/patient/dashboard.php</t>
         </is>
       </c>
       <c r="G49" s="12" t="inlineStr">
@@ -2522,7 +2522,7 @@
       </c>
       <c r="F50" s="15" t="inlineStr">
         <is>
-          <t>Baseline questionnaire submitted successfully. Redirected to: http://localhost/rct-education-web/frontend/patient/procedure_info.php</t>
+          <t>Baseline questionnaire submitted successfully. Redirected to: http://localhost/rct-education-web/frontend_php_backup/patient/procedure_info.php</t>
         </is>
       </c>
       <c r="G50" s="12" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>Educational procedure content viewed successfully. URL: http://localhost/rct-education-web/frontend/patient/education.php?apt=1</t>
+          <t>Educational procedure content viewed successfully. URL: http://localhost/rct-education-web/frontend_php_backup/patient/education.php?apt=1</t>
         </is>
       </c>
       <c r="G51" s="12" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="F52" s="15" t="inlineStr">
         <is>
-          <t>Anxiety levels submitted successfully. Redirected to: http://localhost/rct-education-web/frontend/patient/quiz.php?apt=1</t>
+          <t>Anxiety levels submitted successfully. Redirected to: http://localhost/rct-education-web/frontend_php_backup/patient/quiz.php?apt=1</t>
         </is>
       </c>
       <c r="G52" s="12" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>MCQ Quiz submitted; confirmation modal continue routes correctly. URL: http://localhost/rct-education-web/frontend/patient/dashboard.php</t>
+          <t>MCQ Quiz submitted; confirmation modal continue routes correctly. URL: http://localhost/rct-education-web/frontend_php_backup/patient/dashboard.php</t>
         </is>
       </c>
       <c r="G53" s="12" t="inlineStr">
@@ -3572,7 +3572,7 @@
       </c>
       <c r="F75" s="11" t="inlineStr">
         <is>
-          <t>Loaded patient detail logs view page successfully. URL: http://localhost/rct-education-web/frontend/admin/patient-detail.php?id=57</t>
+          <t>Loaded patient detail logs view page successfully. URL: http://localhost/rct-education-web/frontend_php_backup/admin/patient-detail.php?id=106</t>
         </is>
       </c>
       <c r="G75" s="12" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="F90" s="15" t="inlineStr">
         <is>
-          <t>Language file compiled correctly: No syntax errors detected in c:/xampp/htdocs/rct-education-web/backend/languages/en.php</t>
+          <t>Language file compiled correctly: No syntax errors detected in C:/xampp/htdocs/rct-education-web/backend/languages/en.php</t>
         </is>
       </c>
       <c r="G90" s="12" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="F106" s="15" t="inlineStr">
         <is>
-          <t>DB_HOST defined as localhost in configuration settings.</t>
+          <t>DB_HOST defined correctly in configuration settings.</t>
         </is>
       </c>
       <c r="G106" s="12" t="inlineStr">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="F108" s="15" t="inlineStr">
         <is>
-          <t>Asset bootstrap.min.css exists at: c:\xampp\htdocs\rct-education-web\frontend\assets\css\bootstrap.min.css</t>
+          <t>Asset bootstrap.min.css exists at: C:\xampp\htdocs\rct-education-web\frontend_php_backup\assets\css\bootstrap.min.css</t>
         </is>
       </c>
       <c r="G108" s="12" t="inlineStr">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="F109" s="11" t="inlineStr">
         <is>
-          <t>Asset bootstrap.bundle.min.js exists at: c:\xampp\htdocs\rct-education-web\frontend\assets\js\bootstrap.bundle.min.js</t>
+          <t>Asset bootstrap.bundle.min.js exists at: C:\xampp\htdocs\rct-education-web\frontend_php_backup\assets\js\bootstrap.bundle.min.js</t>
         </is>
       </c>
       <c r="G109" s="12" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="F110" s="15" t="inlineStr">
         <is>
-          <t>Asset style.css exists at: c:\xampp\htdocs\rct-education-web\frontend\assets\css\style.css</t>
+          <t>Asset style.css exists at: C:\xampp\htdocs\rct-education-web\frontend_php_backup\assets\css\style.css</t>
         </is>
       </c>
       <c r="G110" s="12" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="F111" s="11" t="inlineStr">
         <is>
-          <t>Asset script.js exists at: c:\xampp\htdocs\rct-education-web\frontend\assets\js\script.js</t>
+          <t>Asset script.js exists at: C:\xampp\htdocs\rct-education-web\frontend_php_backup\assets\js\script.js</t>
         </is>
       </c>
       <c r="G111" s="12" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="F112" s="15" t="inlineStr">
         <is>
-          <t>Port 80 is active. Apache Web Server is online.</t>
+          <t>Port 80 is active. Web Server is online.</t>
         </is>
       </c>
       <c r="G112" s="12" t="inlineStr">
@@ -5168,7 +5168,7 @@
       </c>
       <c r="F113" s="11" t="inlineStr">
         <is>
-          <t>Port 3306 is active. MySQL Database Engine is online.</t>
+          <t>Port 3306 is active on localhost. Database Engine is online.</t>
         </is>
       </c>
       <c r="G113" s="12" t="inlineStr">

</xml_diff>